<commit_message>
Seed EP/NV/Surgery product names into Evidence Horizon playbook
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ep_monitor/data/evidence_horizon_playbook_template.xlsx
+++ b/ep_monitor/data/evidence_horizon_playbook_template.xlsx
@@ -894,7 +894,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FARAPULSE | Farawave | Farastar | FARAWAVE | FARASTAR | VersaCross</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -912,7 +916,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PulseSelect | Affera | Sphere-9 | Sphere 9 | Arctic Front | DiamondTemp | PVAC</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -930,7 +938,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>EnSite X | EnSite | Volt PFA | Volt | TactiFlex | TactiCath | Advisor HD Grid | Ampere</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -948,7 +960,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FireMagic | Columbus | EasyFinder</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -966,7 +982,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AtriClip | Isolator Synergy | EPi-Sense | cryoICE</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -986,7 +1006,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Biosense Webster | VARIPULSE | CARTO | QDOT | THERMOCOOL | OPTRELL | Octaray</t>
+          <t>Biosense Webster | VARIPULSE | Varipulse | CARTO | QDOT MICRO | QDOT | THERMOCOOL | ThermoCool | OPTRELL | Octaray | OCTARAY | NuVision</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1026,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Solitaire | Pipeline | React | Phenox | Axium</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1024,7 +1048,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Trevo | Neuroform | Surpass | AXS Catalyst | Target</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1042,7 +1070,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Penumbra System | Indigo | Lightning | RED | ACE</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1060,7 +1092,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>WEB | SOFIA | LVIS | HydroSoft | FRED</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1078,7 +1114,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Azur | Soar | PX SLIM</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1098,7 +1138,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Cerenovus | EMBOTRAP | CERENOVUS</t>
+          <t>Cerenovus | CERENOVUS | EMBOTRAP | EMBOTRAP III | Nimbus | TruFill</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1158,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>da Vinci | Ion | da Vinci Xi | da Vinci SP</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1136,7 +1180,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>da Vinci | Ion</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1154,7 +1202,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Hugo | LigaSure | Signia | Sonicision | Tri-Staple</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1172,7 +1224,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Thunderbeat | VISERA | ENDOEYE</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1190,7 +1246,11 @@
           <t>competitor</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Mako | Neptune | 1788</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1210,7 +1270,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Ethicon | OTTAVA | MONARCH | Echelon | Harmonic</t>
+          <t>Ethicon | OTTAVA | MONARCH | Echelon | Harmonic | Enseal | Megadyne</t>
         </is>
       </c>
     </row>

</xml_diff>